<commit_message>
Update monitoring assignment deliverables
</commit_message>
<xml_diff>
--- a/Updated_Data.xlsx
+++ b/Updated_Data.xlsx
@@ -7,115 +7,115 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Clean_Monitoring" sheetId="1" r:id="rId1"/>
-    <sheet name="Clean_Facilities" sheetId="2" r:id="rId2"/>
-    <sheet name="Division_Results" sheetId="3" r:id="rId3"/>
-    <sheet name="District_Comparison" sheetId="4" r:id="rId4"/>
-    <sheet name="Five_Districts" sheetId="5" r:id="rId5"/>
-    <sheet name="Priority_Divisions" sheetId="6" r:id="rId6"/>
-    <sheet name="Priority_Actions" sheetId="7" r:id="rId7"/>
-    <sheet name="Issue_Log" sheetId="8" r:id="rId8"/>
-    <sheet name="Validation_Checks" sheetId="9" r:id="rId9"/>
-    <sheet name="Location_Fixes" sheetId="10" r:id="rId10"/>
-    <sheet name="Facility_Name_Fixes" sheetId="11" r:id="rId11"/>
-    <sheet name="Anomaly_Review" sheetId="12" r:id="rId12"/>
-    <sheet name="Averaging_Windows" sheetId="13" r:id="rId13"/>
+    <sheet name="Clean Monitoring" sheetId="1" r:id="rId1"/>
+    <sheet name="Clean Facilities" sheetId="2" r:id="rId2"/>
+    <sheet name="Division Results" sheetId="3" r:id="rId3"/>
+    <sheet name="District Comparison" sheetId="4" r:id="rId4"/>
+    <sheet name="Five Districts" sheetId="5" r:id="rId5"/>
+    <sheet name="Priority Divisions" sheetId="6" r:id="rId6"/>
+    <sheet name="Priority Actions" sheetId="7" r:id="rId7"/>
+    <sheet name="Issue Log" sheetId="8" r:id="rId8"/>
+    <sheet name="Validation Checks" sheetId="9" r:id="rId9"/>
+    <sheet name="Location Fixes" sheetId="10" r:id="rId10"/>
+    <sheet name="Facility Name Fixes" sheetId="11" r:id="rId11"/>
+    <sheet name="Anomaly Review" sheetId="12" r:id="rId12"/>
+    <sheet name="Averaging Windows" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8316" uniqueCount="960">
-  <si>
-    <t>division</t>
-  </si>
-  <si>
-    <t>district</t>
-  </si>
-  <si>
-    <t>facilities</t>
-  </si>
-  <si>
-    <t>anc_sessions</t>
-  </si>
-  <si>
-    <t>pnc_sessions</t>
-  </si>
-  <si>
-    <t>scanu_sessions</t>
-  </si>
-  <si>
-    <t>general_medicine_sessions</t>
-  </si>
-  <si>
-    <t>general_surgery_sessions</t>
-  </si>
-  <si>
-    <t>ncd_sessions</t>
-  </si>
-  <si>
-    <t>total_patients</t>
-  </si>
-  <si>
-    <t>total_caregivers</t>
-  </si>
-  <si>
-    <t>trainers</t>
-  </si>
-  <si>
-    <t>avg_sessions_week</t>
-  </si>
-  <si>
-    <t>avg_participants_session</t>
-  </si>
-  <si>
-    <t>sessions_vs_target_pct</t>
-  </si>
-  <si>
-    <t>ccp_quality_assessment_coverage_pct</t>
-  </si>
-  <si>
-    <t>source_row</t>
-  </si>
-  <si>
-    <t>division_original</t>
-  </si>
-  <si>
-    <t>district_original</t>
-  </si>
-  <si>
-    <t>division_raw</t>
-  </si>
-  <si>
-    <t>district_raw</t>
-  </si>
-  <si>
-    <t>total_sessions_quarter</t>
-  </si>
-  <si>
-    <t>total_participants</t>
-  </si>
-  <si>
-    <t>calculated_sessions_week</t>
-  </si>
-  <si>
-    <t>calculated_participants_session</t>
-  </si>
-  <si>
-    <t>comparison_district</t>
-  </si>
-  <si>
-    <t>unusual_target_pct</t>
-  </si>
-  <si>
-    <t>unusual_qa_pct</t>
-  </si>
-  <si>
-    <t>unusual_sessions_per_facility</t>
-  </si>
-  <si>
-    <t>unusual_participants_session</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8316" uniqueCount="958">
+  <si>
+    <t>Division</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>Facilities</t>
+  </si>
+  <si>
+    <t>ANC Sessions</t>
+  </si>
+  <si>
+    <t>PNC Sessions</t>
+  </si>
+  <si>
+    <t>SCANU Sessions</t>
+  </si>
+  <si>
+    <t>General Medicine Sessions</t>
+  </si>
+  <si>
+    <t>General Surgery Sessions</t>
+  </si>
+  <si>
+    <t>NCD Sessions</t>
+  </si>
+  <si>
+    <t>Total Patients</t>
+  </si>
+  <si>
+    <t>Total Caregivers</t>
+  </si>
+  <si>
+    <t>Trainers</t>
+  </si>
+  <si>
+    <t>Avg Sessions Week</t>
+  </si>
+  <si>
+    <t>Avg Participants Session</t>
+  </si>
+  <si>
+    <t>Sessions vs Target %</t>
+  </si>
+  <si>
+    <t>CCP Quality Assessment Coverage %</t>
+  </si>
+  <si>
+    <t>Source Row</t>
+  </si>
+  <si>
+    <t>Division Original</t>
+  </si>
+  <si>
+    <t>District Original</t>
+  </si>
+  <si>
+    <t>Division Raw</t>
+  </si>
+  <si>
+    <t>District Raw</t>
+  </si>
+  <si>
+    <t>Total Sessions Quarter</t>
+  </si>
+  <si>
+    <t>Total Participants</t>
+  </si>
+  <si>
+    <t>Calculated Sessions Week</t>
+  </si>
+  <si>
+    <t>Calculated Participants Session</t>
+  </si>
+  <si>
+    <t>Comparison District</t>
+  </si>
+  <si>
+    <t>Unusual Target %</t>
+  </si>
+  <si>
+    <t>Unusual QA %</t>
+  </si>
+  <si>
+    <t>Unusual Sessions Per Facility</t>
+  </si>
+  <si>
+    <t>Unusual Participants Session</t>
   </si>
   <si>
     <t>Barishal</t>
@@ -328,43 +328,43 @@
     <t>Khulna City</t>
   </si>
   <si>
-    <t>active_since</t>
-  </si>
-  <si>
-    <t>facility_type</t>
-  </si>
-  <si>
-    <t>facility_name</t>
-  </si>
-  <si>
-    <t>total_number_of_sessions</t>
-  </si>
-  <si>
-    <t>average_monthly_sessions</t>
-  </si>
-  <si>
-    <t>total_number_of_participants</t>
-  </si>
-  <si>
-    <t>average_monthly_participants</t>
-  </si>
-  <si>
-    <t>facility_type_original</t>
-  </si>
-  <si>
-    <t>facility_name_original</t>
-  </si>
-  <si>
-    <t>implied_months_sessions</t>
-  </si>
-  <si>
-    <t>implied_months_participants</t>
-  </si>
-  <si>
-    <t>average_participants_session</t>
-  </si>
-  <si>
-    <t>unusual_monthly_sessions</t>
+    <t>Active Since</t>
+  </si>
+  <si>
+    <t>Facility Type</t>
+  </si>
+  <si>
+    <t>Facility Name</t>
+  </si>
+  <si>
+    <t>Total Number of Sessions</t>
+  </si>
+  <si>
+    <t>Average Monthly Sessions</t>
+  </si>
+  <si>
+    <t>Total Number of Participants</t>
+  </si>
+  <si>
+    <t>Average Monthly Participants</t>
+  </si>
+  <si>
+    <t>Facility Type Original</t>
+  </si>
+  <si>
+    <t>Facility Name Original</t>
+  </si>
+  <si>
+    <t>Implied Months Sessions</t>
+  </si>
+  <si>
+    <t>Implied Months Participants</t>
+  </si>
+  <si>
+    <t>Average Participants Session</t>
+  </si>
+  <si>
+    <t>Unusual Monthly Sessions</t>
   </si>
   <si>
     <t>Medical College Hospital</t>
@@ -2495,130 +2495,127 @@
     <t>Mother and Child Welfare Centre (MCWC), Mymensingh Sadar, Mymensingh</t>
   </si>
   <si>
-    <t>weighted_target_pct</t>
-  </si>
-  <si>
-    <t>weighted_qa_pct</t>
-  </si>
-  <si>
-    <t>districts</t>
-  </si>
-  <si>
-    <t>sessions</t>
-  </si>
-  <si>
-    <t>participants</t>
-  </si>
-  <si>
-    <t>sessions_per_facility</t>
-  </si>
-  <si>
-    <t>facilities_per_trainer</t>
-  </si>
-  <si>
-    <t>performance_rank</t>
-  </si>
-  <si>
-    <t>monitoring_rows</t>
-  </si>
-  <si>
-    <t>facilities_monitoring</t>
-  </si>
-  <si>
-    <t>reported_quarter_sessions</t>
-  </si>
-  <si>
-    <t>reported_quarter_participants</t>
-  </si>
-  <si>
-    <t>facilities_history</t>
-  </si>
-  <si>
-    <t>expected_quarter_sessions</t>
-  </si>
-  <si>
-    <t>expected_quarter_participants</t>
-  </si>
-  <si>
-    <t>join_status</t>
-  </si>
-  <si>
-    <t>facility_count_gap</t>
-  </si>
-  <si>
-    <t>session_gap</t>
-  </si>
-  <si>
-    <t>session_gap_pct</t>
+    <t>Weighted Target %</t>
+  </si>
+  <si>
+    <t>Weighted QA %</t>
+  </si>
+  <si>
+    <t>Districts</t>
+  </si>
+  <si>
+    <t>Sessions</t>
+  </si>
+  <si>
+    <t>Participants</t>
+  </si>
+  <si>
+    <t>Sessions Per Facility</t>
+  </si>
+  <si>
+    <t>Facilities Per Trainer</t>
+  </si>
+  <si>
+    <t>Performance Rank</t>
+  </si>
+  <si>
+    <t>Monitoring Rows</t>
+  </si>
+  <si>
+    <t>Facilities Monitoring</t>
+  </si>
+  <si>
+    <t>Reported Quarter Sessions</t>
+  </si>
+  <si>
+    <t>Reported Quarter Participants</t>
+  </si>
+  <si>
+    <t>Facilities History</t>
+  </si>
+  <si>
+    <t>Expected Quarter Sessions</t>
+  </si>
+  <si>
+    <t>Expected Quarter Participants</t>
+  </si>
+  <si>
+    <t>Join Status</t>
+  </si>
+  <si>
+    <t>Facility Count Gap</t>
+  </si>
+  <si>
+    <t>Session Gap</t>
+  </si>
+  <si>
+    <t>Session Gap %</t>
   </si>
   <si>
     <t>Matched</t>
   </si>
   <si>
-    <t>volume_quintile</t>
-  </si>
-  <si>
-    <t>absolute_gap_pct</t>
-  </si>
-  <si>
-    <t>assessment</t>
-  </si>
-  <si>
-    <t>hypothesis</t>
+    <t>Volume Quintile</t>
+  </si>
+  <si>
+    <t>Absolute Gap %</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>Hypothesis</t>
   </si>
   <si>
     <t>Does not align</t>
   </si>
   <si>
-    <t>Monitoring includes 2 more facilities, which probably explains part of the higher total. Check the active-facility list and start dates first.</t>
-  </si>
-  <si>
-    <t>Monitoring includes 5 fewer facilities, which probably explains part of the lower total. Check inactive facilities and missing reports first.</t>
-  </si>
-  <si>
-    <t>Totals close; lists differ</t>
-  </si>
-  <si>
-    <t>The totals are close, but monitoring lists 11 facilities and the older file lists 13. The close result may be accidental, so check both facility lists and reporting dates.</t>
-  </si>
-  <si>
-    <t>Facility counts match, so the number of facilities does not explain the higher total. Check whether activity grew, the periods differ, or the older average is no longer current.</t>
-  </si>
-  <si>
-    <t>Monitoring includes 12 more facilities, which probably explains part of the higher total. Check the active-facility list and start dates first.</t>
-  </si>
-  <si>
-    <t>target_risk</t>
-  </si>
-  <si>
-    <t>qa_risk</t>
-  </si>
-  <si>
-    <t>productivity_risk</t>
-  </si>
-  <si>
-    <t>workload_risk</t>
-  </si>
-  <si>
-    <t>scale_risk</t>
-  </si>
-  <si>
-    <t>priority_score</t>
-  </si>
-  <si>
-    <t>Division</t>
-  </si>
-  <si>
-    <t>Why now</t>
-  </si>
-  <si>
-    <t>First practical action</t>
+    <t>Monitoring includes 2 more facilities, which probably explains part of the higher total session frequency. Need to check the active-facility list and start dates first.</t>
+  </si>
+  <si>
+    <t>Monitoring includes 5 fewer facilities, which probably explains part of the lower total session frequency. We should check inactive facilities and missing reports first.</t>
+  </si>
+  <si>
+    <t>Session totals are close</t>
+  </si>
+  <si>
+    <t>The totals are close, but monitoring lists 11 facilities and the older file lists 13. The close result may be accidental, so need to check both facility lists and reporting dates.</t>
+  </si>
+  <si>
+    <t>Facility counts match, so the number of facilities does not explain the higher total session frequency. It is required to check whether activity grew, the periods differ, or the older average is no longer current.</t>
+  </si>
+  <si>
+    <t>Monitoring includes 12 more facilities, which probably explains part of the higher total session frequency. Need to check the active-facility list and start dates first.</t>
+  </si>
+  <si>
+    <t>Target Risk</t>
+  </si>
+  <si>
+    <t>QA Risk</t>
+  </si>
+  <si>
+    <t>Productivity Risk</t>
+  </si>
+  <si>
+    <t>Workload Risk</t>
+  </si>
+  <si>
+    <t>Scale Risk</t>
+  </si>
+  <si>
+    <t>Priority Score</t>
+  </si>
+  <si>
+    <t>Why Now</t>
+  </si>
+  <si>
+    <t>First Practical Action</t>
   </si>
   <si>
     <t>Largest program (145 facilities), lowest target result (80.5%), and 16.7 sessions per facility.</t>
   </si>
   <si>
-    <t>Start with the lowest-target districts, check session totals against registers, and agree a six-week recovery plan with weekly follow-up.</t>
+    <t>Start with the lowest-target districts, need to check session total against registers, and agree a six-week recovery plan with weekly follow-up.</t>
   </si>
   <si>
     <t>Large program (128 facilities), 87.6% target result, and low QA coverage (67.4%).</t>
@@ -2633,7 +2630,7 @@
     <t>Protect the strong session volume while increasing QA checks and rebalancing or clustering trainer support.</t>
   </si>
   <si>
-    <t>issue</t>
+    <t>Issue</t>
   </si>
   <si>
     <t>Frequency</t>
@@ -2645,61 +2642,61 @@
     <t>Misspelled header</t>
   </si>
   <si>
-    <t>Fixed the spelling in the column name; values stayed the same</t>
+    <t>Fixed spelling in the column name</t>
   </si>
   <si>
     <t>Location spelling/punctuation variants</t>
   </si>
   <si>
-    <t>Made spelling, spacing, and punctuation consistent</t>
+    <t>Made spelling, spacing, &amp; punctuation consistent</t>
   </si>
   <si>
     <t>City-vs-district geography</t>
   </si>
   <si>
-    <t>Kept the city rows; used parent districts only when comparing files</t>
+    <t>Kept the city rows &amp; used parent districts when comparing files</t>
   </si>
   <si>
     <t>Facility-name formatting/location variants</t>
   </si>
   <si>
-    <t>Fixed spacing, commas, and clear location spelling errors</t>
+    <t>Fixed spacing, commas, &amp; clear location spelling errors</t>
   </si>
   <si>
     <t>Facility categories vs brief</t>
   </si>
   <si>
-    <t>Kept all 9 types and noted that the brief says 8</t>
+    <t>Kept all 9 identified facility types in the historic data &amp; noted that the brief says 8</t>
   </si>
   <si>
     <t>District facility-count disagreement</t>
   </si>
   <si>
-    <t>Kept both counts and marked the districts that need checking</t>
+    <t>Kept both dataset counts &amp; marked the districts that need checking</t>
   </si>
   <si>
     <t>Unspecified averaging window</t>
   </si>
   <si>
-    <t>Used the given monthly averages and clearly stated the limitation</t>
+    <t>Used the given monthly averages &amp; clearly stated the limitation</t>
   </si>
   <si>
     <t>Unusual monitoring values</t>
   </si>
   <si>
-    <t>Kept the values and marked them for checking</t>
+    <t>Kept the values &amp; marked them for checking</t>
   </si>
   <si>
     <t>Unusual historical values</t>
   </si>
   <si>
-    <t>check</t>
-  </si>
-  <si>
-    <t>failures</t>
-  </si>
-  <si>
-    <t>Numeric parse failures</t>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Failures</t>
+  </si>
+  <si>
+    <t>Numeric conversion failures</t>
   </si>
   <si>
     <t>Missing required values</t>
@@ -2741,16 +2738,16 @@
     <t>Unmatched geographies</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>field</t>
-  </si>
-  <si>
-    <t>original</t>
-  </si>
-  <si>
-    <t>corrected</t>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Original</t>
+  </si>
+  <si>
+    <t>Corrected</t>
   </si>
   <si>
     <t>Monitoring</t>
@@ -2831,16 +2828,13 @@
     <t>Barishal / Bhola</t>
   </si>
   <si>
-    <t>row</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>indicator</t>
-  </si>
-  <si>
-    <t>value</t>
+    <t>Row</t>
+  </si>
+  <si>
+    <t>Indicator</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
   <si>
     <t>Average monthly sessions</t>
@@ -2900,13 +2894,13 @@
     <t>Dhaka / Narayanganj</t>
   </si>
   <si>
-    <t>minimum_implied_months</t>
-  </si>
-  <si>
-    <t>median_implied_months</t>
-  </si>
-  <si>
-    <t>maximum_implied_months</t>
+    <t>Minimum Implied Months</t>
+  </si>
+  <si>
+    <t>Median Implied Months</t>
+  </si>
+  <si>
+    <t>Maximum Implied Months</t>
   </si>
 </sst>
 </file>
@@ -9612,184 +9606,184 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>904</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>905</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>906</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
+        <v>907</v>
+      </c>
+      <c r="B2" t="s">
         <v>908</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>909</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>910</v>
-      </c>
-      <c r="D2" t="s">
-        <v>911</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>907</v>
+      </c>
+      <c r="B3" t="s">
         <v>908</v>
       </c>
-      <c r="B3" t="s">
-        <v>909</v>
-      </c>
       <c r="C3" t="s">
+        <v>911</v>
+      </c>
+      <c r="D3" t="s">
         <v>912</v>
-      </c>
-      <c r="D3" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
+        <v>913</v>
+      </c>
+      <c r="B4" t="s">
+        <v>908</v>
+      </c>
+      <c r="C4" t="s">
         <v>914</v>
       </c>
-      <c r="B4" t="s">
-        <v>909</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>915</v>
-      </c>
-      <c r="D4" t="s">
-        <v>916</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B5" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C5" t="s">
+        <v>916</v>
+      </c>
+      <c r="D5" t="s">
         <v>917</v>
-      </c>
-      <c r="D5" t="s">
-        <v>918</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C6" t="s">
+        <v>918</v>
+      </c>
+      <c r="D6" t="s">
         <v>919</v>
-      </c>
-      <c r="D6" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B7" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C7" t="s">
+        <v>920</v>
+      </c>
+      <c r="D7" t="s">
         <v>921</v>
-      </c>
-      <c r="D7" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B8" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C8" t="s">
+        <v>922</v>
+      </c>
+      <c r="D8" t="s">
         <v>923</v>
-      </c>
-      <c r="D8" t="s">
-        <v>924</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B9" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C9" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="D9" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B10" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C10" t="s">
+        <v>925</v>
+      </c>
+      <c r="D10" t="s">
         <v>926</v>
-      </c>
-      <c r="D10" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B11" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C11" t="s">
+        <v>927</v>
+      </c>
+      <c r="D11" t="s">
         <v>928</v>
-      </c>
-      <c r="D11" t="s">
-        <v>929</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B12" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C12" t="s">
+        <v>929</v>
+      </c>
+      <c r="D12" t="s">
         <v>930</v>
-      </c>
-      <c r="D12" t="s">
-        <v>931</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B13" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C13" t="s">
+        <v>931</v>
+      </c>
+      <c r="D13" t="s">
         <v>932</v>
-      </c>
-      <c r="D13" t="s">
-        <v>933</v>
       </c>
     </row>
   </sheetData>
@@ -9804,13 +9798,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>905</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>906</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -10221,33 +10215,33 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>933</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>934</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>935</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>936</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>937</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B2">
         <v>222</v>
       </c>
       <c r="C2" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="D2" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E2">
         <v>47.777778</v>
@@ -10255,16 +10249,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B3">
         <v>404</v>
       </c>
       <c r="C3" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="D3" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E3">
         <v>39.285714</v>
@@ -10272,16 +10266,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B4">
         <v>555</v>
       </c>
       <c r="C4" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="D4" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E4">
         <v>34</v>
@@ -10289,16 +10283,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B5">
         <v>142</v>
       </c>
       <c r="C5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="D5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E5">
         <v>33.111111</v>
@@ -10306,16 +10300,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B6">
         <v>107</v>
       </c>
       <c r="C6" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="D6" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E6">
         <v>31.25</v>
@@ -10323,16 +10317,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B7">
         <v>379</v>
       </c>
       <c r="C7" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="D7" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E7">
         <v>28</v>
@@ -10340,16 +10334,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B8">
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="D8" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E8">
         <v>27.551724</v>
@@ -10357,16 +10351,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B9">
         <v>235</v>
       </c>
       <c r="C9" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="D9" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E9">
         <v>27.421053</v>
@@ -10374,16 +10368,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B10">
         <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="D10" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E10">
         <v>26.133333</v>
@@ -10391,16 +10385,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B11">
         <v>175</v>
       </c>
       <c r="C11" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D11" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E11">
         <v>25.555556</v>
@@ -10408,16 +10402,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B12">
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="D12" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E12">
         <v>25.416667</v>
@@ -10425,16 +10419,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B13">
         <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="D13" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E13">
         <v>25.227273</v>
@@ -10442,16 +10436,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B14">
         <v>540</v>
       </c>
       <c r="C14" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="D14" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E14">
         <v>24.833333</v>
@@ -10459,16 +10453,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B15">
         <v>262</v>
       </c>
       <c r="C15" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="D15" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E15">
         <v>23.5</v>
@@ -10476,16 +10470,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B16">
         <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="D16" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E16">
         <v>23.235294</v>
@@ -10493,16 +10487,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B17">
         <v>302</v>
       </c>
       <c r="C17" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="D17" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E17">
         <v>23.111111</v>
@@ -10510,16 +10504,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B18">
         <v>416</v>
       </c>
       <c r="C18" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="D18" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E18">
         <v>23</v>
@@ -10527,16 +10521,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B19">
         <v>344</v>
       </c>
       <c r="C19" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D19" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E19">
         <v>22.777778</v>
@@ -10544,16 +10538,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B20">
         <v>217</v>
       </c>
       <c r="C20" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="D20" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E20">
         <v>22.6</v>
@@ -10561,16 +10555,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B21">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="D21" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="E21">
         <v>11.609756</v>
@@ -10578,16 +10572,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B22">
         <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="D22" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E22">
         <v>44.2</v>
@@ -10595,16 +10589,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B23">
         <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="D23" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E23">
         <v>39.6</v>
@@ -10612,16 +10606,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B24">
         <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="D24" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E24">
         <v>38</v>
@@ -10629,16 +10623,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B25">
         <v>19</v>
       </c>
       <c r="C25" t="s">
+        <v>951</v>
+      </c>
+      <c r="D25" t="s">
         <v>953</v>
-      </c>
-      <c r="D25" t="s">
-        <v>955</v>
       </c>
       <c r="E25">
         <v>35.7</v>
@@ -10662,13 +10656,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>955</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>957</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>958</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>959</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -61382,13 +61376,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>859</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>860</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -61396,10 +61390,10 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
+        <v>861</v>
+      </c>
+      <c r="C2" t="s">
         <v>862</v>
-      </c>
-      <c r="C2" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -61407,10 +61401,10 @@
         <v>36</v>
       </c>
       <c r="B3" t="s">
+        <v>863</v>
+      </c>
+      <c r="C3" t="s">
         <v>864</v>
-      </c>
-      <c r="C3" t="s">
-        <v>865</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -61418,10 +61412,10 @@
         <v>30</v>
       </c>
       <c r="B4" t="s">
+        <v>865</v>
+      </c>
+      <c r="C4" t="s">
         <v>866</v>
-      </c>
-      <c r="C4" t="s">
-        <v>867</v>
       </c>
     </row>
   </sheetData>
@@ -61436,112 +61430,112 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>868</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>869</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>870</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B3">
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B5">
         <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B6">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B7">
         <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B8">
         <v>658</v>
       </c>
       <c r="C8" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B10">
         <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
   </sheetData>
@@ -61556,15 +61550,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>887</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>888</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>889</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -61572,7 +61566,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -61580,7 +61574,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -61588,7 +61582,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -61596,7 +61590,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -61604,7 +61598,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -61612,7 +61606,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -61620,7 +61614,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -61628,7 +61622,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -61636,7 +61630,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -61644,7 +61638,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -61652,7 +61646,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -61660,7 +61654,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -61668,7 +61662,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B15">
         <v>0</v>

</xml_diff>